<commit_message>
app funcionando ok- falta eliminar registros
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:U9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46162</v>
+        <v>46164</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
@@ -625,11 +625,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LS1</t>
+          <t>LS2</t>
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46162</v>
+        <v>46164</v>
       </c>
       <c r="C3" t="n">
         <v>2</v>
@@ -683,21 +683,21 @@
         <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>2.07</v>
+        <v>0</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>wewe</t>
+          <t>wewewewewe</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>wewe</t>
+          <t>wewewewewew</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>wewe</t>
+          <t>wewewewewewe</t>
         </is>
       </c>
       <c r="R3" s="1" t="n">
@@ -713,9 +713,531 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>wewewewe</t>
-        </is>
-      </c>
+          <t>wewewewewewewee</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>LS2</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Concentrado Relave</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Planta Conc Relav General</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Celda Columnar 1</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Correa Transportadora</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Lubricación</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Quiebre Stock</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Inmediato 24 h</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0-20</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>wewewewewe</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>wewewewewew</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>wewewewewewe</t>
+        </is>
+      </c>
+      <c r="R4" s="1" t="n">
+        <v>46162</v>
+      </c>
+      <c r="S4" s="1" t="n">
+        <v>46162</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>wewewewewewewee</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LS2</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>46163</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Concentrado Relave</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Planta Conc Relav General</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Celda Columnar 1</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Correa Transportadora</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Lubricación</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Quiebre Stock</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Inmediato 24 h</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0-20</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>wewewewewe</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>wewewewewew</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>wewewewewewe</t>
+        </is>
+      </c>
+      <c r="R5" s="1" t="n">
+        <v>46162</v>
+      </c>
+      <c r="S5" s="1" t="n">
+        <v>46162</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>wewewewewewewee</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LS1</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>46162</v>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Concentrado Relave</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Planta Conc Relav General</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Celda Columnar 1</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Correa Transportadora</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Lubricación</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Quiebre Stock</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Inmediato 24 h</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0-20</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" s="1" t="n">
+        <v>46162</v>
+      </c>
+      <c r="S6" s="1" t="n">
+        <v>46162</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LS2</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>46164</v>
+      </c>
+      <c r="C7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Concentrado Relave</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Planta Conc Relav General</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Celda Columnar 1</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Correa Transportadora</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Lubricación</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Quiebre Stock</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Inmediato 24 h</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0-20</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>wewewewewe</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>wewewewewew</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>wewewewewewe</t>
+        </is>
+      </c>
+      <c r="R7" s="1" t="n">
+        <v>46162</v>
+      </c>
+      <c r="S7" s="1" t="n">
+        <v>46162</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>wewewewewewewee</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LS1</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>46164</v>
+      </c>
+      <c r="C8" t="n">
+        <v>7</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Concentrado Relave</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Planta Conc Relav General</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Celda Columnar 1</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Correa Transportadora</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Lubricación</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Quiebre Stock</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Inmediato 24 h</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0-20</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" s="1" t="n">
+        <v>46162</v>
+      </c>
+      <c r="S8" s="1" t="n">
+        <v>46162</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LS1</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>46164</v>
+      </c>
+      <c r="C9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Concentrado Relave</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Planta Conc Relav General</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Celda Columnar 1</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Correa Transportadora</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Lubricación</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Quiebre Stock</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Inmediato 24 h</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0-20</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" s="1" t="n">
+        <v>46162</v>
+      </c>
+      <c r="S9" s="1" t="n">
+        <v>46162</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
agrego: eliminar registro, actualizar ID y mover ID a primera fila
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -530,11 +530,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LS1</t>
+          <t>LS2</t>
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46164</v>
+        <v>46163</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
@@ -720,11 +720,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LS2</t>
+          <t>LS1</t>
         </is>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46148</v>
+        <v>46169</v>
       </c>
       <c r="C4" t="n">
         <v>3</v>
@@ -780,46 +780,30 @@
       <c r="N4" t="n">
         <v>0</v>
       </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>wewewewewe</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>wewewewewew</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>wewewewewewe</t>
-        </is>
-      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
       <c r="R4" s="1" t="n">
-        <v>46162</v>
+        <v>46169</v>
       </c>
       <c r="S4" s="1" t="n">
-        <v>46162</v>
+        <v>46169</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>wewewewewewewee</t>
-        </is>
-      </c>
+      <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LS2</t>
+          <t>LS1</t>
         </is>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46163</v>
+        <v>46168</v>
       </c>
       <c r="C5" t="n">
         <v>4</v>
@@ -875,369 +859,21 @@
       <c r="N5" t="n">
         <v>0</v>
       </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>wewewewewe</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>wewewewewew</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>wewewewewewe</t>
-        </is>
-      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
       <c r="R5" s="1" t="n">
-        <v>46162</v>
+        <v>46169</v>
       </c>
       <c r="S5" s="1" t="n">
-        <v>46162</v>
+        <v>46169</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>wewewewewewewee</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>LS1</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>46162</v>
-      </c>
-      <c r="C6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Concentrado Relave</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Planta Conc Relav General</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Celda Columnar 1</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Correa Transportadora</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Lubricación</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Quiebre Stock</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Inmediato 24 h</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>0-20</t>
-        </is>
-      </c>
-      <c r="M6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" s="1" t="n">
-        <v>46162</v>
-      </c>
-      <c r="S6" s="1" t="n">
-        <v>46162</v>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>LS2</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>46164</v>
-      </c>
-      <c r="C7" t="n">
-        <v>6</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Concentrado Relave</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Planta Conc Relav General</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Celda Columnar 1</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Correa Transportadora</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Lubricación</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Quiebre Stock</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Inmediato 24 h</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>0-20</t>
-        </is>
-      </c>
-      <c r="M7" t="n">
-        <v>1</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>wewewewewe</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>wewewewewew</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>wewewewewewe</t>
-        </is>
-      </c>
-      <c r="R7" s="1" t="n">
-        <v>46162</v>
-      </c>
-      <c r="S7" s="1" t="n">
-        <v>46162</v>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>wewewewewewewee</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>LS1</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>46164</v>
-      </c>
-      <c r="C8" t="n">
-        <v>7</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Concentrado Relave</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Planta Conc Relav General</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Celda Columnar 1</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Correa Transportadora</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Lubricación</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Quiebre Stock</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Inmediato 24 h</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>0-20</t>
-        </is>
-      </c>
-      <c r="M8" t="n">
-        <v>1</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" s="1" t="n">
-        <v>46162</v>
-      </c>
-      <c r="S8" s="1" t="n">
-        <v>46162</v>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>LS1</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>46164</v>
-      </c>
-      <c r="C9" t="n">
-        <v>8</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Concentrado Relave</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Planta Conc Relav General</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Celda Columnar 1</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Correa Transportadora</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Lubricación</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Quiebre Stock</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Inmediato 24 h</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>0-20</t>
-        </is>
-      </c>
-      <c r="M9" t="n">
-        <v>1</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" s="1" t="n">
-        <v>46162</v>
-      </c>
-      <c r="S9" s="1" t="n">
-        <v>46162</v>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>